<commit_message>
fix: greedy allocation of on calls
</commit_message>
<xml_diff>
--- a/on_call_rota_16people_colored.xlsx
+++ b/on_call_rota_16people_colored.xlsx
@@ -596,11 +596,6 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>UA</t>
@@ -609,6 +604,11 @@
       <c r="P4" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -694,14 +694,14 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -716,14 +716,14 @@
           <t>Wednesday</t>
         </is>
       </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -738,14 +738,14 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -770,7 +770,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="P11" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -831,6 +831,11 @@
           <t>Monday</t>
         </is>
       </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Academic</t>
@@ -844,11 +849,6 @@
       <c r="O14" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="R14" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
           <t>Academic</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -900,11 +900,6 @@
           <t>Academic</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="N16" t="inlineStr">
         <is>
           <t>UA</t>
@@ -913,6 +908,11 @@
       <c r="O16" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
           <t>Academic</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -964,7 +964,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -1040,7 +1040,7 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -1057,7 +1057,7 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr">
+      <c r="R22" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -1074,7 +1074,7 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="M23" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -1091,7 +1091,7 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -1108,6 +1108,11 @@
           <t>Friday</t>
         </is>
       </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="K25" t="inlineStr">
         <is>
           <t>UA</t>
@@ -1116,11 +1121,6 @@
       <c r="M25" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="R25" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -1201,7 +1201,7 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -1223,7 +1223,7 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -1245,6 +1245,11 @@
           <t>Thursday</t>
         </is>
       </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="K31" t="inlineStr">
         <is>
           <t>UA</t>
@@ -1253,11 +1258,6 @@
       <c r="P31" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="R31" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1277,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="O32" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -1343,14 +1343,14 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="K35" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -1375,14 +1375,14 @@
           <t>Tuesday</t>
         </is>
       </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="K36" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -1429,7 +1429,7 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -1471,14 +1471,14 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="K39" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -1584,11 +1584,6 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="I43" t="inlineStr">
         <is>
           <t>UA</t>
@@ -1597,6 +1592,11 @@
       <c r="J43" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="Q43" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -1611,6 +1611,11 @@
           <t>Wednesday</t>
         </is>
       </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>UA</t>
@@ -1619,11 +1624,6 @@
       <c r="J44" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="O44" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="Q45" s="2" t="inlineStr">
+      <c r="P45" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -1670,14 +1670,14 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="J46" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -1736,19 +1736,14 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="F49" t="inlineStr">
         <is>
           <t>UA</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -1763,19 +1758,14 @@
           <t>Tuesday</t>
         </is>
       </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="F50" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="R50" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -1790,19 +1780,14 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="F51" t="inlineStr">
         <is>
           <t>UA</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -1817,19 +1802,14 @@
           <t>Thursday</t>
         </is>
       </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="F52" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="P52" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -1849,14 +1829,9 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1846,7 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="H54" s="3" t="inlineStr">
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>WC SM</t>
         </is>
@@ -1893,7 +1868,7 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>WC SM</t>
         </is>
@@ -1925,12 +1900,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr">
+      <c r="R56" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -1952,11 +1922,6 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
@@ -1979,14 +1944,9 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -2001,19 +1961,14 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="F59" t="inlineStr">
         <is>
           <t>UA</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -2033,14 +1988,14 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr">
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>BH SM</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
         <is>
           <t>BH UHB</t>
-        </is>
-      </c>
-      <c r="P60" t="inlineStr">
-        <is>
-          <t>BH SM</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2059,7 @@
           <t>BH SM</t>
         </is>
       </c>
-      <c r="Q63" t="inlineStr">
+      <c r="L63" t="inlineStr">
         <is>
           <t>BH UHB</t>
         </is>
@@ -2131,11 +2086,6 @@
           <t>On Call</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="M64" t="inlineStr">
         <is>
           <t>UA</t>
@@ -2158,11 +2108,6 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="M65" t="inlineStr">
         <is>
           <t>UA</t>
@@ -2195,11 +2140,6 @@
           <t>On Call</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="M66" t="inlineStr">
         <is>
           <t>UA</t>
@@ -2217,6 +2157,11 @@
           <t>Friday</t>
         </is>
       </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="F67" t="inlineStr">
         <is>
           <t>UA</t>
@@ -2230,11 +2175,6 @@
       <c r="J67" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="L67" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -2259,7 +2199,7 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="G68" s="3" t="inlineStr">
+      <c r="H68" s="3" t="inlineStr">
         <is>
           <t>WC SM</t>
         </is>
@@ -2281,7 +2221,7 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="G69" s="3" t="inlineStr">
+      <c r="H69" s="3" t="inlineStr">
         <is>
           <t>WC SM</t>
         </is>
@@ -2375,6 +2315,11 @@
           <t>UA</t>
         </is>
       </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="M71" t="inlineStr">
         <is>
           <t>UA</t>
@@ -2388,11 +2333,6 @@
       <c r="O71" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="Q71" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -2407,6 +2347,11 @@
           <t>Wednesday</t>
         </is>
       </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="D72" t="inlineStr">
         <is>
           <t>UA</t>
@@ -2425,11 +2370,6 @@
       <c r="J72" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="L72" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -2464,11 +2404,6 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="F73" t="inlineStr">
         <is>
           <t>UA</t>
@@ -2502,6 +2437,11 @@
       <c r="P73" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="Q73" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2476,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="K74" s="2" t="inlineStr">
+      <c r="L74" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -2573,7 +2513,7 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="L75" s="4" t="inlineStr">
+      <c r="K75" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -2595,7 +2535,7 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="L76" s="4" t="inlineStr">
+      <c r="K76" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -2664,6 +2604,11 @@
           <t>Tuesday</t>
         </is>
       </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="F78" t="inlineStr">
         <is>
           <t>UA</t>
@@ -2692,11 +2637,6 @@
       <c r="N78" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="R78" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -2726,7 +2666,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="K79" s="2" t="inlineStr">
+      <c r="L79" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -2748,11 +2688,6 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="F80" t="inlineStr">
         <is>
           <t>UA</t>
@@ -2771,6 +2706,11 @@
       <c r="M80" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="P80" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -2790,11 +2730,6 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="H81" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="I81" t="inlineStr">
         <is>
           <t>UA</t>
@@ -2813,6 +2748,11 @@
       <c r="P81" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="Q81" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2767,7 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="K82" s="4" t="inlineStr">
+      <c r="L82" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -2849,7 +2789,7 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="K83" s="4" t="inlineStr">
+      <c r="L83" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -2881,11 +2821,6 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="M84" t="inlineStr">
         <is>
           <t>UA</t>
@@ -2913,11 +2848,6 @@
           <t>On Call</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="N85" t="inlineStr">
         <is>
           <t>UA</t>
@@ -2935,11 +2865,6 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="M86" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
@@ -2962,12 +2887,7 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="P87" s="2" t="inlineStr">
+      <c r="D87" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -2989,19 +2909,14 @@
           <t>UA</t>
         </is>
       </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="I88" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="Q88" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -3026,7 +2941,7 @@
           <t>WC SM</t>
         </is>
       </c>
-      <c r="M89" s="4" t="inlineStr">
+      <c r="J89" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -3048,7 +2963,7 @@
           <t>WC SM</t>
         </is>
       </c>
-      <c r="M90" s="4" t="inlineStr">
+      <c r="J90" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -3065,12 +2980,12 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
+      <c r="F91" t="inlineStr">
         <is>
           <t>BH SM</t>
         </is>
       </c>
-      <c r="L91" t="inlineStr">
+      <c r="J91" t="inlineStr">
         <is>
           <t>BH UHB</t>
         </is>
@@ -3087,14 +3002,9 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
-      <c r="J92" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -3109,12 +3019,7 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="N93" s="2" t="inlineStr">
+      <c r="C93" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -3131,14 +3036,9 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -3153,14 +3053,14 @@
           <t>Friday</t>
         </is>
       </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="J95" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="P95" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -3219,14 +3119,9 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="H98" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
-      <c r="J98" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -3246,14 +3141,9 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="F99" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
-      <c r="J99" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="R99" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -3268,14 +3158,9 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="I100" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
-      <c r="J100" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -3290,11 +3175,6 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="L101" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
@@ -3312,14 +3192,9 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="D102" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
-      <c r="J102" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3214,7 @@
           <t>WC SM</t>
         </is>
       </c>
-      <c r="K103" s="4" t="inlineStr">
+      <c r="M103" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -3361,7 +3236,7 @@
           <t>WC SM</t>
         </is>
       </c>
-      <c r="K104" s="4" t="inlineStr">
+      <c r="M104" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -3378,12 +3253,7 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="K105" s="2" t="inlineStr">
+      <c r="I105" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -3400,11 +3270,6 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="J106" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
@@ -3422,14 +3287,9 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="G107" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
-      <c r="J107" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -3444,11 +3304,6 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="M108" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
@@ -3476,19 +3331,14 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="E109" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="G109" t="inlineStr">
         <is>
           <t>UA</t>
         </is>
       </c>
-      <c r="J109" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="R109" t="inlineStr">
@@ -3513,7 +3363,7 @@
           <t>WC SM</t>
         </is>
       </c>
-      <c r="L110" s="4" t="inlineStr">
+      <c r="J110" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -3535,7 +3385,7 @@
           <t>WC SM</t>
         </is>
       </c>
-      <c r="L111" s="4" t="inlineStr">
+      <c r="J111" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -3552,12 +3402,12 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr">
+      <c r="C112" t="inlineStr">
         <is>
           <t>BH SM</t>
         </is>
       </c>
-      <c r="K112" t="inlineStr">
+      <c r="I112" t="inlineStr">
         <is>
           <t>BH UHB</t>
         </is>
@@ -3579,16 +3429,16 @@
           <t>UA</t>
         </is>
       </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="G113" t="inlineStr">
         <is>
           <t>UA</t>
         </is>
       </c>
-      <c r="J113" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="O113" t="inlineStr">
         <is>
           <t>UA</t>
@@ -3597,11 +3447,6 @@
       <c r="P113" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="Q113" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -3626,19 +3471,14 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="F114" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="G114" t="inlineStr">
         <is>
           <t>UA</t>
         </is>
       </c>
-      <c r="J114" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="O114" t="inlineStr">
@@ -3673,21 +3513,11 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="E115" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="G115" t="inlineStr">
         <is>
           <t>UA</t>
         </is>
       </c>
-      <c r="J115" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="O115" t="inlineStr">
         <is>
           <t>UA</t>
@@ -3696,6 +3526,11 @@
       <c r="P115" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="Q115" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -3730,12 +3565,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J116" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="M116" s="2" t="inlineStr">
+      <c r="K116" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -3772,7 +3602,7 @@
           <t>WC SM</t>
         </is>
       </c>
-      <c r="Q117" s="4" t="inlineStr">
+      <c r="K117" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -3794,7 +3624,7 @@
           <t>WC SM</t>
         </is>
       </c>
-      <c r="Q118" s="4" t="inlineStr">
+      <c r="K118" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -3811,6 +3641,11 @@
           <t>Monday</t>
         </is>
       </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="G119" t="inlineStr">
         <is>
           <t>UA</t>
@@ -3821,19 +3656,9 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J119" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="Q119" t="inlineStr">
         <is>
           <t>OffRota</t>
-        </is>
-      </c>
-      <c r="R119" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -3848,19 +3673,14 @@
           <t>Tuesday</t>
         </is>
       </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="I120" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="J120" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="L120" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -3885,24 +3705,19 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="D121" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="I121" t="inlineStr">
         <is>
           <t>UA</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="N121" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="P121" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -3927,24 +3742,19 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J122" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="N122" t="inlineStr">
         <is>
           <t>UA</t>
         </is>
       </c>
-      <c r="P122" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="Q122" t="inlineStr">
         <is>
           <t>OffRota</t>
+        </is>
+      </c>
+      <c r="R122" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -3959,17 +3769,12 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="F123" s="2" t="inlineStr">
+      <c r="D123" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="J123" t="inlineStr">
         <is>
           <t>UA</t>
         </is>
@@ -4040,11 +3845,6 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J126" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="K126" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
@@ -4067,14 +3867,9 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="I127" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
-      <c r="J127" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
@@ -4094,12 +3889,7 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="J128" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="N128" s="2" t="inlineStr">
+      <c r="D128" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -4121,14 +3911,9 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C129" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
-      <c r="J129" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="L129" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
@@ -4153,11 +3938,6 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J130" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="Q130" t="inlineStr">
         <is>
           <t>OffRota</t>
@@ -4224,14 +4004,9 @@
           <t>Monday</t>
         </is>
       </c>
-      <c r="H133" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
-      <c r="J133" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
@@ -4251,12 +4026,7 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="J134" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="O134" s="2" t="inlineStr">
+      <c r="H134" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -4278,14 +4048,9 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="F135" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
-      <c r="J135" t="inlineStr">
-        <is>
-          <t>UA</t>
+      <c r="N135" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -4305,24 +4070,19 @@
           <t>Thursday</t>
         </is>
       </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="I136" t="inlineStr">
         <is>
           <t>UA</t>
         </is>
       </c>
-      <c r="J136" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
       <c r="Q136" t="inlineStr">
         <is>
           <t>OffRota</t>
-        </is>
-      </c>
-      <c r="R136" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -4342,19 +4102,14 @@
           <t>UA</t>
         </is>
       </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="I137" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="J137" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="K137" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
@@ -4384,7 +4139,7 @@
           <t>WC SM</t>
         </is>
       </c>
-      <c r="K138" s="4" t="inlineStr">
+      <c r="J138" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -4406,7 +4161,7 @@
           <t>WC SM</t>
         </is>
       </c>
-      <c r="K139" s="4" t="inlineStr">
+      <c r="J139" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -4455,7 +4210,7 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="L141" s="2" t="inlineStr">
+      <c r="O141" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -4509,7 +4264,7 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="N143" s="2" t="inlineStr">
+      <c r="F143" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -4541,7 +4296,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="I144" s="2" t="inlineStr">
+      <c r="L144" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -4568,14 +4323,14 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="J145" s="4" t="inlineStr">
+      <c r="H145" s="3" t="inlineStr">
+        <is>
+          <t>WC SM</t>
+        </is>
+      </c>
+      <c r="L145" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
-        </is>
-      </c>
-      <c r="N145" s="3" t="inlineStr">
-        <is>
-          <t>WC SM</t>
         </is>
       </c>
     </row>
@@ -4590,14 +4345,14 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="J146" s="4" t="inlineStr">
+      <c r="H146" s="3" t="inlineStr">
+        <is>
+          <t>WC SM</t>
+        </is>
+      </c>
+      <c r="L146" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
-        </is>
-      </c>
-      <c r="N146" s="3" t="inlineStr">
-        <is>
-          <t>WC SM</t>
         </is>
       </c>
     </row>
@@ -4617,14 +4372,14 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J147" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="Q147" t="inlineStr">
         <is>
           <t>OffRota</t>
+        </is>
+      </c>
+      <c r="R147" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4399,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="H148" s="2" t="inlineStr">
+      <c r="N148" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -4676,7 +4431,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="I149" s="2" t="inlineStr">
+      <c r="L149" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -4703,14 +4458,14 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C150" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="D150" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="O150" t="inlineStr">
@@ -4745,7 +4500,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="L151" s="2" t="inlineStr">
+      <c r="I151" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -4816,14 +4571,14 @@
           <t>Monday</t>
         </is>
       </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="D154" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="J154" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
       <c r="Q154" t="inlineStr">
@@ -4880,7 +4635,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="P156" s="2" t="inlineStr">
+      <c r="I156" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -4907,7 +4662,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="M157" s="2" t="inlineStr">
+      <c r="J157" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -4929,11 +4684,6 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="C158" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="D158" t="inlineStr">
         <is>
           <t>UA</t>
@@ -4942,6 +4692,11 @@
       <c r="G158" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="Q158" t="inlineStr">
@@ -4961,14 +4716,14 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="C159" s="3" t="inlineStr">
+      <c r="K159" s="4" t="inlineStr">
+        <is>
+          <t>WC UHB</t>
+        </is>
+      </c>
+      <c r="N159" s="3" t="inlineStr">
         <is>
           <t>WC SM</t>
-        </is>
-      </c>
-      <c r="J159" s="4" t="inlineStr">
-        <is>
-          <t>WC UHB</t>
         </is>
       </c>
     </row>
@@ -4983,14 +4738,14 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="C160" s="3" t="inlineStr">
+      <c r="K160" s="4" t="inlineStr">
+        <is>
+          <t>WC UHB</t>
+        </is>
+      </c>
+      <c r="N160" s="3" t="inlineStr">
         <is>
           <t>WC SM</t>
-        </is>
-      </c>
-      <c r="J160" s="4" t="inlineStr">
-        <is>
-          <t>WC UHB</t>
         </is>
       </c>
     </row>
@@ -5010,7 +4765,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J161" s="2" t="inlineStr">
+      <c r="G161" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -5037,11 +4792,6 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="G162" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="N162" t="inlineStr">
         <is>
           <t>UA</t>
@@ -5050,6 +4800,11 @@
       <c r="Q162" t="inlineStr">
         <is>
           <t>OffRota</t>
+        </is>
+      </c>
+      <c r="R162" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -5074,14 +4829,14 @@
           <t>UA</t>
         </is>
       </c>
+      <c r="P163" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="Q163" t="inlineStr">
         <is>
           <t>OffRota</t>
-        </is>
-      </c>
-      <c r="R163" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -5101,14 +4856,14 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="F164" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="I164" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="M164" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="Q164" t="inlineStr">
@@ -5160,12 +4915,12 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="H166" s="3" t="inlineStr">
+      <c r="C166" s="3" t="inlineStr">
         <is>
           <t>WC SM</t>
         </is>
       </c>
-      <c r="O166" s="4" t="inlineStr">
+      <c r="M166" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -5182,12 +4937,12 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="H167" s="3" t="inlineStr">
+      <c r="C167" s="3" t="inlineStr">
         <is>
           <t>WC SM</t>
         </is>
       </c>
-      <c r="O167" s="4" t="inlineStr">
+      <c r="M167" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -5214,7 +4969,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="L168" s="2" t="inlineStr">
+      <c r="K168" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -5246,14 +5001,14 @@
           <t>UA</t>
         </is>
       </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="I169" t="inlineStr">
         <is>
           <t>UA</t>
-        </is>
-      </c>
-      <c r="K169" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
       <c r="Q169" t="inlineStr">
@@ -5300,14 +5055,14 @@
           <t>Thursday</t>
         </is>
       </c>
-      <c r="C171" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="I171" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="L171" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="Q171" t="inlineStr">
@@ -5327,7 +5082,7 @@
           <t>Friday</t>
         </is>
       </c>
-      <c r="J172" s="2" t="inlineStr">
+      <c r="C172" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -5354,7 +5109,7 @@
           <t>WC SM</t>
         </is>
       </c>
-      <c r="J173" s="4" t="inlineStr">
+      <c r="I173" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -5376,7 +5131,7 @@
           <t>WC SM</t>
         </is>
       </c>
-      <c r="J174" s="4" t="inlineStr">
+      <c r="I174" s="4" t="inlineStr">
         <is>
           <t>WC UHB</t>
         </is>
@@ -5447,7 +5202,7 @@
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="J177" s="2" t="inlineStr">
+      <c r="C177" s="2" t="inlineStr">
         <is>
           <t>On Call</t>
         </is>
@@ -5474,6 +5229,11 @@
           <t>Thursday</t>
         </is>
       </c>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
+        </is>
+      </c>
       <c r="N178" t="inlineStr">
         <is>
           <t>UA</t>
@@ -5482,11 +5242,6 @@
       <c r="Q178" t="inlineStr">
         <is>
           <t>OffRota</t>
-        </is>
-      </c>
-      <c r="R178" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
         </is>
       </c>
     </row>
@@ -5506,14 +5261,14 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="H179" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="I179" t="inlineStr">
         <is>
           <t>UA</t>
+        </is>
+      </c>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
       <c r="Q179" t="inlineStr">
@@ -5533,14 +5288,14 @@
           <t>Saturday</t>
         </is>
       </c>
-      <c r="F180" s="3" t="inlineStr">
+      <c r="K180" s="4" t="inlineStr">
+        <is>
+          <t>WC UHB</t>
+        </is>
+      </c>
+      <c r="O180" s="3" t="inlineStr">
         <is>
           <t>WC SM</t>
-        </is>
-      </c>
-      <c r="R180" s="4" t="inlineStr">
-        <is>
-          <t>WC UHB</t>
         </is>
       </c>
     </row>
@@ -5555,14 +5310,14 @@
           <t>Sunday</t>
         </is>
       </c>
-      <c r="F181" s="3" t="inlineStr">
+      <c r="K181" s="4" t="inlineStr">
+        <is>
+          <t>WC UHB</t>
+        </is>
+      </c>
+      <c r="O181" s="3" t="inlineStr">
         <is>
           <t>WC SM</t>
-        </is>
-      </c>
-      <c r="R181" s="4" t="inlineStr">
-        <is>
-          <t>WC UHB</t>
         </is>
       </c>
     </row>
@@ -5604,11 +5359,6 @@
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="F183" s="2" t="inlineStr">
-        <is>
-          <t>On Call</t>
-        </is>
-      </c>
       <c r="I183" t="inlineStr">
         <is>
           <t>UA</t>
@@ -5617,6 +5367,11 @@
       <c r="Q183" t="inlineStr">
         <is>
           <t>OffRota</t>
+        </is>
+      </c>
+      <c r="R183" s="2" t="inlineStr">
+        <is>
+          <t>On Call</t>
         </is>
       </c>
     </row>

</xml_diff>